<commit_message>
Fixed GMM pipeline encoding issues, updated Streamlit UI, and cleaned up unnecessary redundant scripts
</commit_message>
<xml_diff>
--- a/Output_results.xlsx
+++ b/Output_results.xlsx
@@ -593,13 +593,13 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>19.3361</v>
+        <v>33.3333</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>20.3165</v>
+        <v>33.3333</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>20.5808</v>
+        <v>33.3333</v>
       </c>
       <c r="L6" s="5" t="n"/>
       <c r="M6" s="6" t="inlineStr">
@@ -676,13 +676,13 @@
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>20.4712</v>
+        <v>33.3333</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>21.1009</v>
+        <v>33.3333</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>21.1035</v>
+        <v>33.3333</v>
       </c>
       <c r="L10" s="5" t="n"/>
       <c r="N10" s="12" t="inlineStr">
@@ -754,13 +754,13 @@
         </is>
       </c>
       <c r="C14" s="5" t="n">
-        <v>20.1977</v>
+        <v>33.3333</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>20.297</v>
+        <v>33.3333</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>20.1662</v>
+        <v>33.3333</v>
       </c>
       <c r="L14" s="5" t="n"/>
     </row>
@@ -827,13 +827,13 @@
         </is>
       </c>
       <c r="C18" s="5" t="n">
-        <v>19.5263</v>
+        <v>33.3333</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>20.1349</v>
+        <v>33.3333</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>20.1805</v>
+        <v>33.3333</v>
       </c>
       <c r="L18" s="5" t="n"/>
     </row>
@@ -900,13 +900,13 @@
         </is>
       </c>
       <c r="C22" s="5" t="n">
-        <v>18.9138</v>
+        <v>33.3334</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>20.0745</v>
+        <v>33.3333</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>19.9415</v>
+        <v>33.3334</v>
       </c>
       <c r="L22" s="5" t="n"/>
     </row>
@@ -973,13 +973,13 @@
         </is>
       </c>
       <c r="C26" s="5" t="n">
-        <v>18.6003</v>
+        <v>33.3333</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>19.5948</v>
+        <v>33.3334</v>
       </c>
       <c r="I26" s="5" t="n">
-        <v>19.531</v>
+        <v>33.3333</v>
       </c>
       <c r="L26" s="5" t="n"/>
     </row>
@@ -1046,13 +1046,13 @@
         </is>
       </c>
       <c r="C30" s="5" t="n">
-        <v>19.8565</v>
+        <v>33.3333</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>20.6268</v>
+        <v>33.3333</v>
       </c>
       <c r="I30" s="5" t="n">
-        <v>21.0688</v>
+        <v>33.3333</v>
       </c>
       <c r="L30" s="5" t="n"/>
     </row>
@@ -1119,13 +1119,13 @@
         </is>
       </c>
       <c r="C34" s="5" t="n">
-        <v>20.8859</v>
+        <v>33.3334</v>
       </c>
       <c r="F34" s="5" t="n">
-        <v>21.8905</v>
+        <v>33.3333</v>
       </c>
       <c r="I34" s="5" t="n">
-        <v>21.8235</v>
+        <v>33.3333</v>
       </c>
       <c r="L34" s="5" t="n"/>
     </row>
@@ -1192,13 +1192,13 @@
         </is>
       </c>
       <c r="C38" s="5" t="n">
-        <v>20.6663</v>
+        <v>33.3333</v>
       </c>
       <c r="F38" s="5" t="n">
-        <v>20.836</v>
+        <v>33.3333</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>21.0186</v>
+        <v>33.3333</v>
       </c>
       <c r="L38" s="5" t="n"/>
     </row>
@@ -1265,13 +1265,13 @@
         </is>
       </c>
       <c r="C42" s="5" t="n">
-        <v>20.2606</v>
+        <v>33.3333</v>
       </c>
       <c r="F42" s="5" t="n">
-        <v>20.8648</v>
+        <v>33.3333</v>
       </c>
       <c r="I42" s="5" t="n">
-        <v>20.9695</v>
+        <v>33.3333</v>
       </c>
       <c r="L42" s="5" t="n"/>
     </row>
@@ -1338,13 +1338,13 @@
         </is>
       </c>
       <c r="C46" s="5" t="n">
-        <v>21.4246</v>
+        <v>33.3333</v>
       </c>
       <c r="F46" s="5" t="n">
-        <v>22.2032</v>
+        <v>33.3333</v>
       </c>
       <c r="I46" s="5" t="n">
-        <v>22.2502</v>
+        <v>33.3333</v>
       </c>
       <c r="L46" s="5" t="n"/>
     </row>
@@ -1411,13 +1411,13 @@
         </is>
       </c>
       <c r="C50" s="5" t="n">
-        <v>20.9266</v>
+        <v>33.3333</v>
       </c>
       <c r="F50" s="5" t="n">
-        <v>22.0047</v>
+        <v>33.3334</v>
       </c>
       <c r="I50" s="5" t="n">
-        <v>21.7604</v>
+        <v>33.3333</v>
       </c>
       <c r="L50" s="5" t="n"/>
     </row>
@@ -1484,13 +1484,13 @@
         </is>
       </c>
       <c r="C54" s="5" t="n">
-        <v>19.7917</v>
+        <v>33.3333</v>
       </c>
       <c r="F54" s="5" t="n">
-        <v>20.591</v>
+        <v>33.3333</v>
       </c>
       <c r="I54" s="5" t="n">
-        <v>20.1258</v>
+        <v>33.3333</v>
       </c>
       <c r="L54" s="5" t="n"/>
     </row>
@@ -1557,13 +1557,13 @@
         </is>
       </c>
       <c r="C58" s="5" t="n">
-        <v>20.5969</v>
+        <v>33.3333</v>
       </c>
       <c r="F58" s="5" t="n">
-        <v>21.5882</v>
+        <v>33.3333</v>
       </c>
       <c r="I58" s="5" t="n">
-        <v>21.699</v>
+        <v>33.3333</v>
       </c>
       <c r="L58" s="5" t="n"/>
     </row>
@@ -1630,13 +1630,13 @@
         </is>
       </c>
       <c r="C62" s="5" t="n">
-        <v>20.0134</v>
+        <v>33.3333</v>
       </c>
       <c r="F62" s="5" t="n">
-        <v>20.9274</v>
+        <v>33.3333</v>
       </c>
       <c r="I62" s="5" t="n">
-        <v>20.6506</v>
+        <v>33.3333</v>
       </c>
       <c r="L62" s="5" t="n"/>
     </row>
@@ -1703,13 +1703,13 @@
         </is>
       </c>
       <c r="C66" s="5" t="n">
-        <v>21.1544</v>
+        <v>33.3333</v>
       </c>
       <c r="F66" s="5" t="n">
-        <v>22.4395</v>
+        <v>33.3333</v>
       </c>
       <c r="I66" s="5" t="n">
-        <v>22.0344</v>
+        <v>33.3333</v>
       </c>
       <c r="L66" s="5" t="n"/>
     </row>
@@ -1776,13 +1776,13 @@
         </is>
       </c>
       <c r="C70" s="5" t="n">
-        <v>19.9451</v>
+        <v>33.3333</v>
       </c>
       <c r="F70" s="5" t="n">
-        <v>21.0974</v>
+        <v>33.3333</v>
       </c>
       <c r="I70" s="5" t="n">
-        <v>20.5761</v>
+        <v>33.3334</v>
       </c>
       <c r="L70" s="5" t="n"/>
     </row>
@@ -1849,13 +1849,13 @@
         </is>
       </c>
       <c r="C74" s="5" t="n">
-        <v>20.8567</v>
+        <v>33.3333</v>
       </c>
       <c r="F74" s="5" t="n">
-        <v>21.1754</v>
+        <v>33.3333</v>
       </c>
       <c r="I74" s="5" t="n">
-        <v>21.217</v>
+        <v>33.3333</v>
       </c>
       <c r="L74" s="5" t="n"/>
     </row>
@@ -1922,13 +1922,13 @@
         </is>
       </c>
       <c r="C78" s="5" t="n">
-        <v>20.6592</v>
+        <v>33.3333</v>
       </c>
       <c r="F78" s="5" t="n">
-        <v>21.5079</v>
+        <v>33.3333</v>
       </c>
       <c r="I78" s="5" t="n">
-        <v>21.3071</v>
+        <v>33.3333</v>
       </c>
       <c r="L78" s="5" t="n"/>
     </row>
@@ -1995,13 +1995,13 @@
         </is>
       </c>
       <c r="C82" s="5" t="n">
-        <v>20.8408</v>
+        <v>33.3333</v>
       </c>
       <c r="F82" s="5" t="n">
-        <v>21.1872</v>
+        <v>33.3333</v>
       </c>
       <c r="I82" s="5" t="n">
-        <v>21.2312</v>
+        <v>33.3333</v>
       </c>
       <c r="L82" s="5" t="n"/>
     </row>
@@ -2068,13 +2068,13 @@
         </is>
       </c>
       <c r="C86" s="5" t="n">
-        <v>20.1814</v>
+        <v>33.3333</v>
       </c>
       <c r="F86" s="5" t="n">
-        <v>20.3385</v>
+        <v>33.3333</v>
       </c>
       <c r="I86" s="5" t="n">
-        <v>20.3721</v>
+        <v>33.3333</v>
       </c>
       <c r="L86" s="5" t="n"/>
     </row>
@@ -2141,13 +2141,13 @@
         </is>
       </c>
       <c r="C90" s="5" t="n">
-        <v>19.3076</v>
+        <v>33.3333</v>
       </c>
       <c r="F90" s="5" t="n">
-        <v>19.1093</v>
+        <v>33.3333</v>
       </c>
       <c r="I90" s="5" t="n">
-        <v>19.2124</v>
+        <v>33.3333</v>
       </c>
       <c r="L90" s="5" t="n"/>
     </row>
@@ -2214,13 +2214,13 @@
         </is>
       </c>
       <c r="C94" s="5" t="n">
-        <v>20.0235</v>
+        <v>33.3333</v>
       </c>
       <c r="F94" s="5" t="n">
-        <v>21.282</v>
+        <v>33.3333</v>
       </c>
       <c r="I94" s="5" t="n">
-        <v>21.635</v>
+        <v>33.3333</v>
       </c>
       <c r="L94" s="5" t="n"/>
     </row>
@@ -2287,13 +2287,13 @@
         </is>
       </c>
       <c r="C98" s="5" t="n">
-        <v>21.0417</v>
+        <v>33.3333</v>
       </c>
       <c r="F98" s="5" t="n">
-        <v>22.1443</v>
+        <v>33.3333</v>
       </c>
       <c r="I98" s="5" t="n">
-        <v>22.23</v>
+        <v>33.3333</v>
       </c>
       <c r="L98" s="5" t="n"/>
     </row>
@@ -2360,13 +2360,13 @@
         </is>
       </c>
       <c r="C102" s="5" t="n">
-        <v>20.4202</v>
+        <v>33.3333</v>
       </c>
       <c r="F102" s="5" t="n">
-        <v>22.2222</v>
+        <v>33.3333</v>
       </c>
       <c r="I102" s="5" t="n">
-        <v>21.4928</v>
+        <v>33.3333</v>
       </c>
       <c r="L102" s="5" t="n"/>
     </row>
@@ -2433,13 +2433,13 @@
         </is>
       </c>
       <c r="C106" s="5" t="n">
-        <v>20.6237</v>
+        <v>33.3333</v>
       </c>
       <c r="F106" s="5" t="n">
-        <v>21.8292</v>
+        <v>33.3333</v>
       </c>
       <c r="I106" s="5" t="n">
-        <v>21.7436</v>
+        <v>33.3333</v>
       </c>
       <c r="L106" s="5" t="n"/>
     </row>
@@ -2506,13 +2506,13 @@
         </is>
       </c>
       <c r="C110" s="5" t="n">
-        <v>21.0154</v>
+        <v>33.3333</v>
       </c>
       <c r="F110" s="5" t="n">
-        <v>21.2263</v>
+        <v>33.3334</v>
       </c>
       <c r="I110" s="5" t="n">
-        <v>21.2492</v>
+        <v>33.3333</v>
       </c>
       <c r="L110" s="5" t="n"/>
     </row>
@@ -2579,13 +2579,13 @@
         </is>
       </c>
       <c r="C114" s="5" t="n">
-        <v>20.9199</v>
+        <v>33.3334</v>
       </c>
       <c r="F114" s="5" t="n">
-        <v>22.1181</v>
+        <v>33.3333</v>
       </c>
       <c r="I114" s="5" t="n">
-        <v>22.0637</v>
+        <v>33.3333</v>
       </c>
       <c r="L114" s="5" t="n"/>
     </row>
@@ -2652,13 +2652,13 @@
         </is>
       </c>
       <c r="C118" s="5" t="n">
-        <v>21.6307</v>
+        <v>33.3333</v>
       </c>
       <c r="F118" s="5" t="n">
-        <v>22.5115</v>
+        <v>33.3333</v>
       </c>
       <c r="I118" s="5" t="n">
-        <v>22.5608</v>
+        <v>33.3333</v>
       </c>
       <c r="L118" s="5" t="n"/>
     </row>
@@ -2725,13 +2725,13 @@
         </is>
       </c>
       <c r="C122" s="5" t="n">
-        <v>20.8149</v>
+        <v>33.3333</v>
       </c>
       <c r="F122" s="5" t="n">
-        <v>21.5337</v>
+        <v>33.3333</v>
       </c>
       <c r="I122" s="5" t="n">
-        <v>21.5857</v>
+        <v>33.3333</v>
       </c>
       <c r="L122" s="5" t="n"/>
     </row>
@@ -2798,13 +2798,13 @@
         </is>
       </c>
       <c r="C126" s="5" t="n">
-        <v>19.3451</v>
+        <v>33.3333</v>
       </c>
       <c r="F126" s="5" t="n">
-        <v>20.1113</v>
+        <v>33.3333</v>
       </c>
       <c r="I126" s="5" t="n">
-        <v>20.1142</v>
+        <v>33.3334</v>
       </c>
       <c r="L126" s="5" t="n"/>
     </row>
@@ -2871,13 +2871,13 @@
         </is>
       </c>
       <c r="C130" s="5" t="n">
-        <v>20.5226</v>
+        <v>33.3333</v>
       </c>
       <c r="F130" s="5" t="n">
-        <v>20.8378</v>
+        <v>33.3333</v>
       </c>
       <c r="I130" s="5" t="n">
-        <v>21.0087</v>
+        <v>33.3333</v>
       </c>
       <c r="L130" s="5" t="n"/>
     </row>
@@ -2944,13 +2944,13 @@
         </is>
       </c>
       <c r="C134" s="5" t="n">
-        <v>19.5683</v>
+        <v>33.3333</v>
       </c>
       <c r="F134" s="5" t="n">
-        <v>19.8249</v>
+        <v>33.3334</v>
       </c>
       <c r="I134" s="5" t="n">
-        <v>19.9758</v>
+        <v>33.3334</v>
       </c>
       <c r="L134" s="5" t="n"/>
     </row>
@@ -3017,13 +3017,13 @@
         </is>
       </c>
       <c r="C138" s="5" t="n">
-        <v>21.2891</v>
+        <v>33.3333</v>
       </c>
       <c r="F138" s="5" t="n">
-        <v>22.7838</v>
+        <v>33.3334</v>
       </c>
       <c r="I138" s="5" t="n">
-        <v>22.768</v>
+        <v>33.3333</v>
       </c>
       <c r="L138" s="5" t="n"/>
     </row>
@@ -3090,13 +3090,13 @@
         </is>
       </c>
       <c r="C142" s="5" t="n">
-        <v>21.6986</v>
+        <v>33.3333</v>
       </c>
       <c r="F142" s="5" t="n">
-        <v>21.9344</v>
+        <v>33.3333</v>
       </c>
       <c r="I142" s="5" t="n">
-        <v>22.4572</v>
+        <v>33.3333</v>
       </c>
       <c r="L142" s="5" t="n"/>
     </row>
@@ -3163,13 +3163,13 @@
         </is>
       </c>
       <c r="C146" s="5" t="n">
-        <v>20.1065</v>
+        <v>33.3333</v>
       </c>
       <c r="F146" s="5" t="n">
-        <v>21.2782</v>
+        <v>33.3333</v>
       </c>
       <c r="I146" s="5" t="n">
-        <v>21.2282</v>
+        <v>33.3333</v>
       </c>
       <c r="L146" s="5" t="n"/>
     </row>
@@ -3236,13 +3236,13 @@
         </is>
       </c>
       <c r="C150" s="5" t="n">
-        <v>21.3132</v>
+        <v>33.3333</v>
       </c>
       <c r="F150" s="5" t="n">
-        <v>21.8585</v>
+        <v>33.3333</v>
       </c>
       <c r="I150" s="5" t="n">
-        <v>21.8408</v>
+        <v>33.3333</v>
       </c>
       <c r="L150" s="5" t="n"/>
     </row>
@@ -3309,13 +3309,13 @@
         </is>
       </c>
       <c r="C154" s="5" t="n">
-        <v>21.4271</v>
+        <v>33.3334</v>
       </c>
       <c r="F154" s="5" t="n">
-        <v>22.967</v>
+        <v>33.3333</v>
       </c>
       <c r="I154" s="5" t="n">
-        <v>22.2364</v>
+        <v>33.3333</v>
       </c>
       <c r="L154" s="5" t="n"/>
     </row>
@@ -3382,13 +3382,13 @@
         </is>
       </c>
       <c r="C158" s="5" t="n">
-        <v>19.6818</v>
+        <v>33.3334</v>
       </c>
       <c r="F158" s="5" t="n">
-        <v>19.9196</v>
+        <v>33.3333</v>
       </c>
       <c r="I158" s="5" t="n">
-        <v>19.9272</v>
+        <v>33.3333</v>
       </c>
       <c r="L158" s="5" t="n"/>
     </row>
@@ -3455,13 +3455,13 @@
         </is>
       </c>
       <c r="C162" s="5" t="n">
-        <v>21.552</v>
+        <v>33.3333</v>
       </c>
       <c r="F162" s="5" t="n">
-        <v>23.377</v>
+        <v>33.3333</v>
       </c>
       <c r="I162" s="5" t="n">
-        <v>23.336</v>
+        <v>33.3333</v>
       </c>
       <c r="L162" s="5" t="n"/>
     </row>
@@ -3528,13 +3528,13 @@
         </is>
       </c>
       <c r="C166" s="5" t="n">
-        <v>20.0358</v>
+        <v>33.3333</v>
       </c>
       <c r="F166" s="5" t="n">
-        <v>20.4666</v>
+        <v>33.3333</v>
       </c>
       <c r="I166" s="5" t="n">
-        <v>19.6589</v>
+        <v>33.3333</v>
       </c>
       <c r="L166" s="5" t="n"/>
     </row>
@@ -3601,13 +3601,13 @@
         </is>
       </c>
       <c r="C170" s="5" t="n">
-        <v>21.1816</v>
+        <v>33.3333</v>
       </c>
       <c r="F170" s="5" t="n">
-        <v>21.6655</v>
+        <v>33.3333</v>
       </c>
       <c r="I170" s="5" t="n">
-        <v>21.6655</v>
+        <v>33.3333</v>
       </c>
       <c r="L170" s="5" t="n"/>
     </row>
@@ -3674,13 +3674,13 @@
         </is>
       </c>
       <c r="C174" s="5" t="n">
-        <v>19.2628</v>
+        <v>33.3333</v>
       </c>
       <c r="F174" s="5" t="n">
-        <v>19.0269</v>
+        <v>33.3333</v>
       </c>
       <c r="I174" s="5" t="n">
-        <v>18.8741</v>
+        <v>33.3333</v>
       </c>
       <c r="L174" s="5" t="n"/>
     </row>
@@ -3747,13 +3747,13 @@
         </is>
       </c>
       <c r="C178" s="5" t="n">
-        <v>20.9576</v>
+        <v>33.3333</v>
       </c>
       <c r="F178" s="5" t="n">
-        <v>21.834</v>
+        <v>33.3333</v>
       </c>
       <c r="I178" s="5" t="n">
-        <v>21.8204</v>
+        <v>33.3333</v>
       </c>
       <c r="L178" s="5" t="n"/>
     </row>
@@ -3820,13 +3820,13 @@
         </is>
       </c>
       <c r="C182" s="5" t="n">
-        <v>21.2595</v>
+        <v>33.3334</v>
       </c>
       <c r="F182" s="5" t="n">
-        <v>22.2605</v>
+        <v>33.3333</v>
       </c>
       <c r="I182" s="5" t="n">
-        <v>22.7843</v>
+        <v>33.3333</v>
       </c>
       <c r="L182" s="5" t="n"/>
     </row>
@@ -3893,13 +3893,13 @@
         </is>
       </c>
       <c r="C186" s="5" t="n">
-        <v>19.5772</v>
+        <v>33.3333</v>
       </c>
       <c r="F186" s="5" t="n">
-        <v>20.2282</v>
+        <v>33.3333</v>
       </c>
       <c r="I186" s="5" t="n">
-        <v>20.2507</v>
+        <v>33.3333</v>
       </c>
       <c r="L186" s="5" t="n"/>
     </row>
@@ -3966,13 +3966,13 @@
         </is>
       </c>
       <c r="C190" s="5" t="n">
-        <v>22.7622</v>
+        <v>33.3334</v>
       </c>
       <c r="F190" s="5" t="n">
-        <v>22.0893</v>
+        <v>33.3333</v>
       </c>
       <c r="I190" s="5" t="n">
-        <v>23.0533</v>
+        <v>33.3333</v>
       </c>
       <c r="L190" s="5" t="n"/>
     </row>
@@ -4039,13 +4039,13 @@
         </is>
       </c>
       <c r="C194" s="5" t="n">
-        <v>20.8704</v>
+        <v>33.3333</v>
       </c>
       <c r="F194" s="5" t="n">
-        <v>20.4301</v>
+        <v>33.3333</v>
       </c>
       <c r="I194" s="5" t="n">
-        <v>20.4521</v>
+        <v>33.3333</v>
       </c>
       <c r="L194" s="5" t="n"/>
     </row>
@@ -4112,13 +4112,13 @@
         </is>
       </c>
       <c r="C198" s="5" t="n">
-        <v>21.7972</v>
+        <v>33.3334</v>
       </c>
       <c r="F198" s="5" t="n">
-        <v>21.9173</v>
+        <v>33.3333</v>
       </c>
       <c r="I198" s="5" t="n">
-        <v>21.7865</v>
+        <v>33.3333</v>
       </c>
       <c r="L198" s="5" t="n"/>
     </row>
@@ -4185,13 +4185,13 @@
         </is>
       </c>
       <c r="C202" s="5" t="n">
-        <v>21.4016</v>
+        <v>33.3333</v>
       </c>
       <c r="F202" s="5" t="n">
-        <v>22.6804</v>
+        <v>33.3334</v>
       </c>
       <c r="I202" s="5" t="n">
-        <v>22.6485</v>
+        <v>33.3334</v>
       </c>
       <c r="L202" s="5" t="n"/>
     </row>
@@ -4922,13 +4922,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>27.4957</v>
+        <v>48.6451</v>
       </c>
       <c r="E4" t="n">
-        <v>20.4317</v>
+        <v>37.6748</v>
       </c>
       <c r="F4" t="n">
-        <v>10.0809</v>
+        <v>13.6801</v>
       </c>
     </row>
     <row r="5">
@@ -4938,13 +4938,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>26.4535</v>
+        <v>45.4701</v>
       </c>
       <c r="E5" t="n">
-        <v>22.7713</v>
+        <v>41.3675</v>
       </c>
       <c r="F5" t="n">
-        <v>11.7248</v>
+        <v>13.1624</v>
       </c>
     </row>
     <row r="6">
@@ -4954,13 +4954,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>26.3258</v>
+        <v>45.4395</v>
       </c>
       <c r="E6" t="n">
-        <v>23.4848</v>
+        <v>41.6252</v>
       </c>
       <c r="F6" t="n">
-        <v>11.9318</v>
+        <v>12.9353</v>
       </c>
     </row>
     <row r="7">
@@ -4975,13 +4975,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>22.0711</v>
+        <v>36.5337</v>
       </c>
       <c r="E7" t="n">
-        <v>25.548</v>
+        <v>42.5187</v>
       </c>
       <c r="F7" t="n">
-        <v>13.7944</v>
+        <v>20.9476</v>
       </c>
     </row>
     <row r="8">
@@ -4991,13 +4991,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>18.3486</v>
+        <v>30.1205</v>
       </c>
       <c r="E8" t="n">
-        <v>25.1376</v>
+        <v>42.1687</v>
       </c>
       <c r="F8" t="n">
-        <v>19.8165</v>
+        <v>27.7108</v>
       </c>
     </row>
     <row r="9">
@@ -5007,13 +5007,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>19.6246</v>
+        <v>32.1229</v>
       </c>
       <c r="E9" t="n">
-        <v>24.9147</v>
+        <v>41.6201</v>
       </c>
       <c r="F9" t="n">
-        <v>18.7713</v>
+        <v>26.257</v>
       </c>
     </row>
     <row r="10">
@@ -5028,13 +5028,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>25.6163</v>
+        <v>43.2916</v>
       </c>
       <c r="E10" t="n">
-        <v>26.9025</v>
+        <v>46.6905</v>
       </c>
       <c r="F10" t="n">
-        <v>8.074299999999999</v>
+        <v>10.0179</v>
       </c>
     </row>
     <row r="11">
@@ -5044,13 +5044,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>24.9505</v>
+        <v>42.1405</v>
       </c>
       <c r="E11" t="n">
-        <v>26.0396</v>
+        <v>45.4849</v>
       </c>
       <c r="F11" t="n">
-        <v>9.901</v>
+        <v>12.3746</v>
       </c>
     </row>
     <row r="12">
@@ -5060,13 +5060,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>24.3528</v>
+        <v>41.7618</v>
       </c>
       <c r="E12" t="n">
-        <v>26.4621</v>
+        <v>46.0033</v>
       </c>
       <c r="F12" t="n">
-        <v>9.6836</v>
+        <v>12.2349</v>
       </c>
     </row>
     <row r="13">
@@ -5081,13 +5081,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>26.8293</v>
+        <v>44.7912</v>
       </c>
       <c r="E13" t="n">
-        <v>24.9661</v>
+        <v>45.5385</v>
       </c>
       <c r="F13" t="n">
-        <v>6.7835</v>
+        <v>9.670299999999999</v>
       </c>
     </row>
     <row r="14">
@@ -5097,13 +5097,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>28.815</v>
+        <v>47.2167</v>
       </c>
       <c r="E14" t="n">
-        <v>23.9017</v>
+        <v>43.0417</v>
       </c>
       <c r="F14" t="n">
-        <v>7.6879</v>
+        <v>9.7416</v>
       </c>
     </row>
     <row r="15">
@@ -5113,13 +5113,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>29.285</v>
+        <v>47.7928</v>
       </c>
       <c r="E15" t="n">
-        <v>23.265</v>
+        <v>41.8468</v>
       </c>
       <c r="F15" t="n">
-        <v>7.9916</v>
+        <v>10.3604</v>
       </c>
     </row>
     <row r="16">
@@ -5134,13 +5134,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>23.1415</v>
+        <v>41.5009</v>
       </c>
       <c r="E16" t="n">
-        <v>24.8195</v>
+        <v>45.6894</v>
       </c>
       <c r="F16" t="n">
-        <v>8.7805</v>
+        <v>12.8098</v>
       </c>
     </row>
     <row r="17">
@@ -5150,13 +5150,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>23.9106</v>
+        <v>42.3892</v>
       </c>
       <c r="E17" t="n">
-        <v>27.0391</v>
+        <v>45.4721</v>
       </c>
       <c r="F17" t="n">
-        <v>9.2737</v>
+        <v>12.1387</v>
       </c>
     </row>
     <row r="18">
@@ -5166,13 +5166,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>24.1493</v>
+        <v>42.8843</v>
       </c>
       <c r="E18" t="n">
-        <v>27.0033</v>
+        <v>45.5408</v>
       </c>
       <c r="F18" t="n">
-        <v>8.671799999999999</v>
+        <v>11.575</v>
       </c>
     </row>
     <row r="19">
@@ -5187,13 +5187,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>24.615</v>
+        <v>45.0094</v>
       </c>
       <c r="E19" t="n">
-        <v>20.7392</v>
+        <v>38.8418</v>
       </c>
       <c r="F19" t="n">
-        <v>10.4466</v>
+        <v>16.1488</v>
       </c>
     </row>
     <row r="20">
@@ -5203,13 +5203,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>22.1273</v>
+        <v>39.8973</v>
       </c>
       <c r="E20" t="n">
-        <v>22.6021</v>
+        <v>40.411</v>
       </c>
       <c r="F20" t="n">
-        <v>14.0551</v>
+        <v>19.6918</v>
       </c>
     </row>
     <row r="21">
@@ -5219,13 +5219,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>21.9824</v>
+        <v>39.9421</v>
       </c>
       <c r="E21" t="n">
-        <v>23.5811</v>
+        <v>41.9682</v>
       </c>
       <c r="F21" t="n">
-        <v>13.0296</v>
+        <v>18.0897</v>
       </c>
     </row>
     <row r="22">
@@ -5240,13 +5240,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>26.4043</v>
+        <v>45.7588</v>
       </c>
       <c r="E22" t="n">
-        <v>23.8816</v>
+        <v>41.8927</v>
       </c>
       <c r="F22" t="n">
-        <v>9.2836</v>
+        <v>12.3485</v>
       </c>
     </row>
     <row r="23">
@@ -5256,13 +5256,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>26.1753</v>
+        <v>46.9933</v>
       </c>
       <c r="E23" t="n">
-        <v>24.1423</v>
+        <v>41.6481</v>
       </c>
       <c r="F23" t="n">
-        <v>11.5629</v>
+        <v>11.3586</v>
       </c>
     </row>
     <row r="24">
@@ -5272,13 +5272,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>25.6242</v>
+        <v>45.4955</v>
       </c>
       <c r="E24" t="n">
-        <v>24.7043</v>
+        <v>41.2162</v>
       </c>
       <c r="F24" t="n">
-        <v>12.8778</v>
+        <v>13.2883</v>
       </c>
     </row>
     <row r="25">
@@ -5293,13 +5293,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>32.5736</v>
+        <v>50.5114</v>
       </c>
       <c r="E25" t="n">
-        <v>23.5624</v>
+        <v>39.5455</v>
       </c>
       <c r="F25" t="n">
-        <v>6.5217</v>
+        <v>9.943199999999999</v>
       </c>
     </row>
     <row r="26">
@@ -5309,13 +5309,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>30.7463</v>
+        <v>47.0126</v>
       </c>
       <c r="E26" t="n">
-        <v>25.4726</v>
+        <v>38.9937</v>
       </c>
       <c r="F26" t="n">
-        <v>9.4527</v>
+        <v>13.9937</v>
       </c>
     </row>
     <row r="27">
@@ -5325,13 +5325,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>31.1348</v>
+        <v>47.9263</v>
       </c>
       <c r="E27" t="n">
-        <v>24.9273</v>
+        <v>38.2488</v>
       </c>
       <c r="F27" t="n">
-        <v>9.408300000000001</v>
+        <v>13.8249</v>
       </c>
     </row>
     <row r="28">
@@ -5346,13 +5346,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>25.5146</v>
+        <v>41.2207</v>
       </c>
       <c r="E28" t="n">
-        <v>25.5417</v>
+        <v>42.7245</v>
       </c>
       <c r="F28" t="n">
-        <v>10.9426</v>
+        <v>16.0548</v>
       </c>
     </row>
     <row r="29">
@@ -5362,13 +5362,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>24.8886</v>
+        <v>39.7317</v>
       </c>
       <c r="E29" t="n">
-        <v>25.9707</v>
+        <v>43.8596</v>
       </c>
       <c r="F29" t="n">
-        <v>11.6486</v>
+        <v>16.4087</v>
       </c>
     </row>
     <row r="30">
@@ -5378,13 +5378,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>24.5337</v>
+        <v>39.2157</v>
       </c>
       <c r="E30" t="n">
-        <v>25.8967</v>
+        <v>43.3679</v>
       </c>
       <c r="F30" t="n">
-        <v>12.6255</v>
+        <v>17.4164</v>
       </c>
     </row>
     <row r="31">
@@ -5399,13 +5399,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>24.9948</v>
+        <v>43.7717</v>
       </c>
       <c r="E31" t="n">
-        <v>27.9268</v>
+        <v>45.5115</v>
       </c>
       <c r="F31" t="n">
-        <v>7.8603</v>
+        <v>10.7168</v>
       </c>
     </row>
     <row r="32">
@@ -5415,13 +5415,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>23.6788</v>
+        <v>40.4063</v>
       </c>
       <c r="E32" t="n">
-        <v>29.3068</v>
+        <v>46.5011</v>
       </c>
       <c r="F32" t="n">
-        <v>9.6088</v>
+        <v>13.0926</v>
       </c>
     </row>
     <row r="33">
@@ -5431,13 +5431,13 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>23.7028</v>
+        <v>40.0839</v>
       </c>
       <c r="E33" t="n">
-        <v>29.5964</v>
+        <v>46.7996</v>
       </c>
       <c r="F33" t="n">
-        <v>9.6092</v>
+        <v>13.1165</v>
       </c>
     </row>
     <row r="34">
@@ -5452,13 +5452,13 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>29.3047</v>
+        <v>53.8803</v>
       </c>
       <c r="E34" t="n">
-        <v>26.571</v>
+        <v>41.2417</v>
       </c>
       <c r="F34" t="n">
-        <v>8.398099999999999</v>
+        <v>4.878</v>
       </c>
     </row>
     <row r="35">
@@ -5468,13 +5468,13 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>31.1073</v>
+        <v>55.3846</v>
       </c>
       <c r="E35" t="n">
-        <v>26.8836</v>
+        <v>41.4201</v>
       </c>
       <c r="F35" t="n">
-        <v>8.6187</v>
+        <v>3.1953</v>
       </c>
     </row>
     <row r="36">
@@ -5484,13 +5484,13 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>30.8611</v>
+        <v>54.8942</v>
       </c>
       <c r="E36" t="n">
-        <v>26.7128</v>
+        <v>41.4021</v>
       </c>
       <c r="F36" t="n">
-        <v>9.176600000000001</v>
+        <v>3.7037</v>
       </c>
     </row>
     <row r="37">
@@ -5505,13 +5505,13 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>25.6478</v>
+        <v>48.6976</v>
       </c>
       <c r="E37" t="n">
-        <v>26.384</v>
+        <v>43.6014</v>
       </c>
       <c r="F37" t="n">
-        <v>10.7479</v>
+        <v>7.701</v>
       </c>
     </row>
     <row r="38">
@@ -5521,13 +5521,13 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>27.2242</v>
+        <v>49.0849</v>
       </c>
       <c r="E38" t="n">
-        <v>28.6477</v>
+        <v>45.9235</v>
       </c>
       <c r="F38" t="n">
-        <v>10.1423</v>
+        <v>4.9917</v>
       </c>
     </row>
     <row r="39">
@@ -5537,13 +5537,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>27.6284</v>
+        <v>50</v>
       </c>
       <c r="E39" t="n">
-        <v>27.6284</v>
+        <v>44.8012</v>
       </c>
       <c r="F39" t="n">
-        <v>10.0244</v>
+        <v>5.1988</v>
       </c>
     </row>
     <row r="40">
@@ -5558,13 +5558,13 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>27.0673</v>
+        <v>52.9635</v>
       </c>
       <c r="E40" t="n">
-        <v>23.149</v>
+        <v>39.0232</v>
       </c>
       <c r="F40" t="n">
-        <v>9.1587</v>
+        <v>8.013299999999999</v>
       </c>
     </row>
     <row r="41">
@@ -5574,13 +5574,13 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>28.0267</v>
+        <v>52.8233</v>
       </c>
       <c r="E41" t="n">
-        <v>23.8322</v>
+        <v>38.0692</v>
       </c>
       <c r="F41" t="n">
-        <v>9.914199999999999</v>
+        <v>9.1075</v>
       </c>
     </row>
     <row r="42">
@@ -5590,13 +5590,13 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>27.7358</v>
+        <v>53.211</v>
       </c>
       <c r="E42" t="n">
-        <v>23.8679</v>
+        <v>37.7982</v>
       </c>
       <c r="F42" t="n">
-        <v>8.7736</v>
+        <v>8.9908</v>
       </c>
     </row>
     <row r="43">
@@ -5611,13 +5611,13 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>24.6387</v>
+        <v>44.7979</v>
       </c>
       <c r="E43" t="n">
-        <v>27.3176</v>
+        <v>45.6594</v>
       </c>
       <c r="F43" t="n">
-        <v>9.834300000000001</v>
+        <v>9.5427</v>
       </c>
     </row>
     <row r="44">
@@ -5627,13 +5627,13 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>26.5335</v>
+        <v>47.7807</v>
       </c>
       <c r="E44" t="n">
-        <v>28.9586</v>
+        <v>45.4308</v>
       </c>
       <c r="F44" t="n">
-        <v>9.272500000000001</v>
+        <v>6.7885</v>
       </c>
     </row>
     <row r="45">
@@ -5643,13 +5643,13 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>26.5928</v>
+        <v>47.3552</v>
       </c>
       <c r="E45" t="n">
-        <v>29.2244</v>
+        <v>46.0957</v>
       </c>
       <c r="F45" t="n">
-        <v>9.2798</v>
+        <v>6.5491</v>
       </c>
     </row>
     <row r="46">
@@ -5664,13 +5664,13 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>24.8935</v>
+        <v>48.3284</v>
       </c>
       <c r="E46" t="n">
-        <v>26.8238</v>
+        <v>44.9853</v>
       </c>
       <c r="F46" t="n">
-        <v>8.322900000000001</v>
+        <v>6.6863</v>
       </c>
     </row>
     <row r="47">
@@ -5680,13 +5680,13 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>25.7101</v>
+        <v>48.9301</v>
       </c>
       <c r="E47" t="n">
-        <v>27.4581</v>
+        <v>46.3623</v>
       </c>
       <c r="F47" t="n">
-        <v>9.614000000000001</v>
+        <v>4.7076</v>
       </c>
     </row>
     <row r="48">
@@ -5696,13 +5696,13 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>25.5148</v>
+        <v>51.0018</v>
       </c>
       <c r="E48" t="n">
-        <v>26.1415</v>
+        <v>44.0801</v>
       </c>
       <c r="F48" t="n">
-        <v>10.2954</v>
+        <v>4.918</v>
       </c>
     </row>
     <row r="49">
@@ -5717,13 +5717,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>24.3082</v>
+        <v>48.5</v>
       </c>
       <c r="E49" t="n">
-        <v>28.5629</v>
+        <v>43.8125</v>
       </c>
       <c r="F49" t="n">
-        <v>10.5921</v>
+        <v>7.6875</v>
       </c>
     </row>
     <row r="50">
@@ -5733,13 +5733,13 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>22.067</v>
+        <v>47.4542</v>
       </c>
       <c r="E50" t="n">
-        <v>33.4264</v>
+        <v>45.0102</v>
       </c>
       <c r="F50" t="n">
-        <v>11.825</v>
+        <v>7.5356</v>
       </c>
     </row>
     <row r="51">
@@ -5749,13 +5749,13 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>21.5023</v>
+        <v>47.4684</v>
       </c>
       <c r="E51" t="n">
-        <v>32.3944</v>
+        <v>44.7257</v>
       </c>
       <c r="F51" t="n">
-        <v>12.2066</v>
+        <v>7.8059</v>
       </c>
     </row>
     <row r="52">
@@ -5770,13 +5770,13 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>21.9104</v>
+        <v>47.4889</v>
       </c>
       <c r="E52" t="n">
-        <v>26.6478</v>
+        <v>47.2346</v>
       </c>
       <c r="F52" t="n">
-        <v>11.277</v>
+        <v>5.2765</v>
       </c>
     </row>
     <row r="53">
@@ -5786,13 +5786,13 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>21.0201</v>
+        <v>46.7532</v>
       </c>
       <c r="E53" t="n">
-        <v>27.357</v>
+        <v>46.3822</v>
       </c>
       <c r="F53" t="n">
-        <v>14.915</v>
+        <v>6.8646</v>
       </c>
     </row>
     <row r="54">
@@ -5802,13 +5802,13 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>20.4586</v>
+        <v>45.9916</v>
       </c>
       <c r="E54" t="n">
-        <v>28.1305</v>
+        <v>47.2574</v>
       </c>
       <c r="F54" t="n">
-        <v>13.1393</v>
+        <v>6.7511</v>
       </c>
     </row>
     <row r="55">
@@ -5823,13 +5823,13 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>26.229</v>
+        <v>50.2427</v>
       </c>
       <c r="E55" t="n">
-        <v>21.9664</v>
+        <v>40.8981</v>
       </c>
       <c r="F55" t="n">
-        <v>14.3746</v>
+        <v>8.8592</v>
       </c>
     </row>
     <row r="56">
@@ -5839,13 +5839,13 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>26.9663</v>
+        <v>52.3729</v>
       </c>
       <c r="E56" t="n">
-        <v>19.9654</v>
+        <v>37.7966</v>
       </c>
       <c r="F56" t="n">
-        <v>16.5946</v>
+        <v>9.830500000000001</v>
       </c>
     </row>
     <row r="57">
@@ -5855,13 +5855,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>27.0616</v>
+        <v>52.5157</v>
       </c>
       <c r="E57" t="n">
-        <v>20.0961</v>
+        <v>37.8931</v>
       </c>
       <c r="F57" t="n">
-        <v>16.4932</v>
+        <v>9.591200000000001</v>
       </c>
     </row>
     <row r="58">
@@ -5876,13 +5876,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>29.6943</v>
+        <v>53.6783</v>
       </c>
       <c r="E58" t="n">
-        <v>23.3624</v>
+        <v>37.9052</v>
       </c>
       <c r="F58" t="n">
-        <v>8.9208</v>
+        <v>8.416499999999999</v>
       </c>
     </row>
     <row r="59">
@@ -5892,13 +5892,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>29.7444</v>
+        <v>53.0303</v>
       </c>
       <c r="E59" t="n">
-        <v>26.0263</v>
+        <v>38.7879</v>
       </c>
       <c r="F59" t="n">
-        <v>8.7529</v>
+        <v>8.181800000000001</v>
       </c>
     </row>
     <row r="60">
@@ -5908,13 +5908,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>29.0063</v>
+        <v>52.9307</v>
       </c>
       <c r="E60" t="n">
-        <v>25.6938</v>
+        <v>38.7211</v>
       </c>
       <c r="F60" t="n">
-        <v>9.2211</v>
+        <v>8.348100000000001</v>
       </c>
     </row>
     <row r="61">
@@ -5929,13 +5929,13 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>27.2504</v>
+        <v>50.6051</v>
       </c>
       <c r="E61" t="n">
-        <v>27.607</v>
+        <v>44.6885</v>
       </c>
       <c r="F61" t="n">
-        <v>7.6649</v>
+        <v>4.7064</v>
       </c>
     </row>
     <row r="62">
@@ -5945,13 +5945,13 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>26.4892</v>
+        <v>49.4238</v>
       </c>
       <c r="E62" t="n">
-        <v>28.1369</v>
+        <v>45.0704</v>
       </c>
       <c r="F62" t="n">
-        <v>8.9354</v>
+        <v>5.5058</v>
       </c>
     </row>
     <row r="63">
@@ -5961,13 +5961,13 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>26.2563</v>
+        <v>48.8491</v>
       </c>
       <c r="E63" t="n">
-        <v>29.4598</v>
+        <v>46.4194</v>
       </c>
       <c r="F63" t="n">
-        <v>7.9774</v>
+        <v>4.7315</v>
       </c>
     </row>
     <row r="64">
@@ -5982,13 +5982,13 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>25.9578</v>
+        <v>49.9276</v>
       </c>
       <c r="E64" t="n">
-        <v>23.6305</v>
+        <v>39.9421</v>
       </c>
       <c r="F64" t="n">
-        <v>10.956</v>
+        <v>10.1302</v>
       </c>
     </row>
     <row r="65">
@@ -5998,13 +5998,13 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>23.3001</v>
+        <v>45.4376</v>
       </c>
       <c r="E65" t="n">
-        <v>25.1133</v>
+        <v>42.0857</v>
       </c>
       <c r="F65" t="n">
-        <v>12.602</v>
+        <v>12.4767</v>
       </c>
     </row>
     <row r="66">
@@ -6014,13 +6014,13 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>24.2195</v>
+        <v>47.3581</v>
       </c>
       <c r="E66" t="n">
-        <v>25.1656</v>
+        <v>41.2916</v>
       </c>
       <c r="F66" t="n">
-        <v>11.7313</v>
+        <v>11.3503</v>
       </c>
     </row>
     <row r="67">
@@ -6035,13 +6035,13 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>22.5986</v>
+        <v>47.8707</v>
       </c>
       <c r="E67" t="n">
-        <v>24.2255</v>
+        <v>38.5839</v>
       </c>
       <c r="F67" t="n">
-        <v>11.0987</v>
+        <v>13.5454</v>
       </c>
     </row>
     <row r="68">
@@ -6051,13 +6051,13 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>20.5668</v>
+        <v>45.328</v>
       </c>
       <c r="E68" t="n">
-        <v>23.9676</v>
+        <v>37.3757</v>
       </c>
       <c r="F68" t="n">
-        <v>12.7935</v>
+        <v>17.2962</v>
       </c>
     </row>
     <row r="69">
@@ -6067,13 +6067,13 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>20.5418</v>
+        <v>45.1673</v>
       </c>
       <c r="E69" t="n">
-        <v>23.8525</v>
+        <v>36.9888</v>
       </c>
       <c r="F69" t="n">
-        <v>13.243</v>
+        <v>17.8439</v>
       </c>
     </row>
     <row r="70">
@@ -6088,13 +6088,13 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>26.5234</v>
+        <v>51.1923</v>
       </c>
       <c r="E70" t="n">
-        <v>23.3483</v>
+        <v>44.7839</v>
       </c>
       <c r="F70" t="n">
-        <v>10.1988</v>
+        <v>4.0238</v>
       </c>
     </row>
     <row r="71">
@@ -6104,13 +6104,13 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>27.4038</v>
+        <v>51.1682</v>
       </c>
       <c r="E71" t="n">
-        <v>22.7885</v>
+        <v>43.9252</v>
       </c>
       <c r="F71" t="n">
-        <v>13.6538</v>
+        <v>4.9065</v>
       </c>
     </row>
     <row r="72">
@@ -6120,13 +6120,13 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>29.1755</v>
+        <v>52.5</v>
       </c>
       <c r="E72" t="n">
-        <v>23.9958</v>
+        <v>44</v>
       </c>
       <c r="F72" t="n">
-        <v>11.7336</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="73">
@@ -6141,13 +6141,13 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>27.5</v>
+        <v>55.0799</v>
       </c>
       <c r="E73" t="n">
-        <v>26.7935</v>
+        <v>39.8402</v>
       </c>
       <c r="F73" t="n">
-        <v>8.8315</v>
+        <v>5.0799</v>
       </c>
     </row>
     <row r="74">
@@ -6157,13 +6157,13 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>28.5047</v>
+        <v>56.564</v>
       </c>
       <c r="E74" t="n">
-        <v>29.0498</v>
+        <v>39.222</v>
       </c>
       <c r="F74" t="n">
-        <v>8.878500000000001</v>
+        <v>4.2139</v>
       </c>
     </row>
     <row r="75">
@@ -6173,13 +6173,13 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>28.2123</v>
+        <v>56.4964</v>
       </c>
       <c r="E75" t="n">
-        <v>29.1201</v>
+        <v>39.562</v>
       </c>
       <c r="F75" t="n">
-        <v>9.3575</v>
+        <v>3.9416</v>
       </c>
     </row>
     <row r="76">
@@ -6194,13 +6194,13 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>26.0688</v>
+        <v>49.8729</v>
       </c>
       <c r="E76" t="n">
-        <v>25.2093</v>
+        <v>42.161</v>
       </c>
       <c r="F76" t="n">
-        <v>9.9824</v>
+        <v>7.9661</v>
       </c>
     </row>
     <row r="77">
@@ -6210,13 +6210,13 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>26.4368</v>
+        <v>46.2766</v>
       </c>
       <c r="E77" t="n">
-        <v>30.0766</v>
+        <v>46.6312</v>
       </c>
       <c r="F77" t="n">
-        <v>10.1533</v>
+        <v>7.0922</v>
       </c>
     </row>
     <row r="78">
@@ -6226,13 +6226,13 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>25.8094</v>
+        <v>46.6216</v>
       </c>
       <c r="E78" t="n">
-        <v>30.036</v>
+        <v>46.4527</v>
       </c>
       <c r="F78" t="n">
-        <v>8.633100000000001</v>
+        <v>6.9257</v>
       </c>
     </row>
     <row r="79">
@@ -6247,13 +6247,13 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>25.6057</v>
+        <v>49.5259</v>
       </c>
       <c r="E79" t="n">
-        <v>27.9911</v>
+        <v>44.1284</v>
       </c>
       <c r="F79" t="n">
-        <v>8.2743</v>
+        <v>6.3457</v>
       </c>
     </row>
     <row r="80">
@@ -6263,13 +6263,13 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>27.5456</v>
+        <v>51.6393</v>
       </c>
       <c r="E80" t="n">
-        <v>28.403</v>
+        <v>42.623</v>
       </c>
       <c r="F80" t="n">
-        <v>9.539099999999999</v>
+        <v>5.7377</v>
       </c>
     </row>
     <row r="81">
@@ -6279,13 +6279,13 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>27.0769</v>
+        <v>50.7843</v>
       </c>
       <c r="E81" t="n">
-        <v>28.1026</v>
+        <v>42.549</v>
       </c>
       <c r="F81" t="n">
-        <v>10.0513</v>
+        <v>6.6667</v>
       </c>
     </row>
     <row r="82">
@@ -6300,13 +6300,13 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>26.4873</v>
+        <v>51.1465</v>
       </c>
       <c r="E82" t="n">
-        <v>25.3024</v>
+        <v>42.5537</v>
       </c>
       <c r="F82" t="n">
-        <v>11.2565</v>
+        <v>6.2998</v>
       </c>
     </row>
     <row r="83">
@@ -6316,13 +6316,13 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>25.0233</v>
+        <v>49.4297</v>
       </c>
       <c r="E83" t="n">
-        <v>27.1242</v>
+        <v>44.7719</v>
       </c>
       <c r="F83" t="n">
-        <v>11.5313</v>
+        <v>5.7985</v>
       </c>
     </row>
     <row r="84">
@@ -6332,13 +6332,13 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>25.0907</v>
+        <v>49.6303</v>
       </c>
       <c r="E84" t="n">
-        <v>27.0871</v>
+        <v>44.732</v>
       </c>
       <c r="F84" t="n">
-        <v>11.5699</v>
+        <v>5.6377</v>
       </c>
     </row>
     <row r="85">
@@ -6353,13 +6353,13 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>24.4974</v>
+        <v>51.4931</v>
       </c>
       <c r="E85" t="n">
-        <v>26.4736</v>
+        <v>42.2433</v>
       </c>
       <c r="F85" t="n">
-        <v>11.7888</v>
+        <v>6.2637</v>
       </c>
     </row>
     <row r="86">
@@ -6369,13 +6369,13 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>26.25</v>
+        <v>50</v>
       </c>
       <c r="E86" t="n">
-        <v>28.4375</v>
+        <v>43.1535</v>
       </c>
       <c r="F86" t="n">
-        <v>11.6667</v>
+        <v>6.8465</v>
       </c>
     </row>
     <row r="87">
@@ -6385,13 +6385,13 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>25.247</v>
+        <v>50.9259</v>
       </c>
       <c r="E87" t="n">
-        <v>28.8694</v>
+        <v>43.5185</v>
       </c>
       <c r="F87" t="n">
-        <v>12.0746</v>
+        <v>5.5556</v>
       </c>
     </row>
     <row r="88">
@@ -6406,13 +6406,13 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>27.2893</v>
+        <v>50.3192</v>
       </c>
       <c r="E88" t="n">
-        <v>27.4719</v>
+        <v>41.2652</v>
       </c>
       <c r="F88" t="n">
-        <v>10.1308</v>
+        <v>8.4156</v>
       </c>
     </row>
     <row r="89">
@@ -6422,13 +6422,13 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>31.0008</v>
+        <v>53.7178</v>
       </c>
       <c r="E89" t="n">
-        <v>26.5256</v>
+        <v>39.4537</v>
       </c>
       <c r="F89" t="n">
-        <v>10.0081</v>
+        <v>6.8285</v>
       </c>
     </row>
     <row r="90">
@@ -6438,13 +6438,13 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>31.2296</v>
+        <v>54.7667</v>
       </c>
       <c r="E90" t="n">
-        <v>26.6594</v>
+        <v>37.7282</v>
       </c>
       <c r="F90" t="n">
-        <v>9.7933</v>
+        <v>7.5051</v>
       </c>
     </row>
     <row r="91">
@@ -6459,13 +6459,13 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>27.9627</v>
+        <v>53.2829</v>
       </c>
       <c r="E91" t="n">
-        <v>24.8196</v>
+        <v>40.9069</v>
       </c>
       <c r="F91" t="n">
-        <v>9.6624</v>
+        <v>5.8101</v>
       </c>
     </row>
     <row r="92">
@@ -6475,13 +6475,13 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>26.6974</v>
+        <v>51.0578</v>
       </c>
       <c r="E92" t="n">
-        <v>23.6651</v>
+        <v>40.7616</v>
       </c>
       <c r="F92" t="n">
-        <v>14.2386</v>
+        <v>8.1805</v>
       </c>
     </row>
     <row r="93">
@@ -6491,13 +6491,13 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>26.3387</v>
+        <v>50.3311</v>
       </c>
       <c r="E93" t="n">
-        <v>24.7821</v>
+        <v>41.8543</v>
       </c>
       <c r="F93" t="n">
-        <v>13.6364</v>
+        <v>7.8146</v>
       </c>
     </row>
     <row r="94">
@@ -6512,13 +6512,13 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>26.1094</v>
+        <v>55.3484</v>
       </c>
       <c r="E94" t="n">
-        <v>21.0685</v>
+        <v>37.1933</v>
       </c>
       <c r="F94" t="n">
-        <v>10.8574</v>
+        <v>7.4583</v>
       </c>
     </row>
     <row r="95">
@@ -6528,13 +6528,13 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>27.4711</v>
+        <v>55.5249</v>
       </c>
       <c r="E95" t="n">
-        <v>22.208</v>
+        <v>38.3978</v>
       </c>
       <c r="F95" t="n">
-        <v>10.6547</v>
+        <v>6.0773</v>
       </c>
     </row>
     <row r="96">
@@ -6544,13 +6544,13 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>27.5398</v>
+        <v>55.5556</v>
       </c>
       <c r="E96" t="n">
-        <v>22.7662</v>
+        <v>38.8889</v>
       </c>
       <c r="F96" t="n">
-        <v>10.0367</v>
+        <v>5.5556</v>
       </c>
     </row>
     <row r="97">
@@ -6565,13 +6565,13 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>24.4742</v>
+        <v>48.5256</v>
       </c>
       <c r="E97" t="n">
-        <v>26.8642</v>
+        <v>45.9615</v>
       </c>
       <c r="F97" t="n">
-        <v>10.2294</v>
+        <v>5.5128</v>
       </c>
     </row>
     <row r="98">
@@ -6581,13 +6581,13 @@
         </is>
       </c>
       <c r="D98" t="n">
-        <v>25.6771</v>
+        <v>50.9132</v>
       </c>
       <c r="E98" t="n">
-        <v>27.4106</v>
+        <v>44.2922</v>
       </c>
       <c r="F98" t="n">
-        <v>9.425800000000001</v>
+        <v>4.7945</v>
       </c>
     </row>
     <row r="99">
@@ -6597,13 +6597,13 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>25.5511</v>
+        <v>50.2092</v>
       </c>
       <c r="E99" t="n">
-        <v>28.2565</v>
+        <v>45.3975</v>
       </c>
       <c r="F99" t="n">
-        <v>9.218400000000001</v>
+        <v>4.3933</v>
       </c>
     </row>
     <row r="100">
@@ -6618,13 +6618,13 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>24.8319</v>
+        <v>52.4422</v>
       </c>
       <c r="E100" t="n">
-        <v>22.4658</v>
+        <v>41.6452</v>
       </c>
       <c r="F100" t="n">
-        <v>11.4072</v>
+        <v>5.9126</v>
       </c>
     </row>
     <row r="101">
@@ -6634,13 +6634,13 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>25.7974</v>
+        <v>52.2353</v>
       </c>
       <c r="E101" t="n">
-        <v>22.6079</v>
+        <v>41.8824</v>
       </c>
       <c r="F101" t="n">
-        <v>11.0694</v>
+        <v>5.8824</v>
       </c>
     </row>
     <row r="102">
@@ -6650,13 +6650,13 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>25.748</v>
+        <v>53.0806</v>
       </c>
       <c r="E102" t="n">
-        <v>22.7561</v>
+        <v>40.9953</v>
       </c>
       <c r="F102" t="n">
-        <v>11.4234</v>
+        <v>5.9242</v>
       </c>
     </row>
     <row r="103">
@@ -6671,13 +6671,13 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>28.3882</v>
+        <v>47.2011</v>
       </c>
       <c r="E103" t="n">
-        <v>29.0923</v>
+        <v>46.3472</v>
       </c>
       <c r="F103" t="n">
-        <v>6.3867</v>
+        <v>6.4516</v>
       </c>
     </row>
     <row r="104">
@@ -6687,13 +6687,13 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>29.4712</v>
+        <v>42.1769</v>
       </c>
       <c r="E104" t="n">
-        <v>30.5599</v>
+        <v>49.932</v>
       </c>
       <c r="F104" t="n">
-        <v>8.320399999999999</v>
+        <v>7.8912</v>
       </c>
     </row>
     <row r="105">
@@ -6703,13 +6703,13 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>29.7007</v>
+        <v>42.6273</v>
       </c>
       <c r="E105" t="n">
-        <v>30.3914</v>
+        <v>49.5979</v>
       </c>
       <c r="F105" t="n">
-        <v>8.2118</v>
+        <v>7.7748</v>
       </c>
     </row>
     <row r="106">
@@ -6724,13 +6724,13 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>27.1756</v>
+        <v>48.2286</v>
       </c>
       <c r="E106" t="n">
-        <v>26.3588</v>
+        <v>44.0571</v>
       </c>
       <c r="F106" t="n">
-        <v>11.5614</v>
+        <v>7.7143</v>
       </c>
     </row>
     <row r="107">
@@ -6740,13 +6740,13 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>26.7703</v>
+        <v>46.9136</v>
       </c>
       <c r="E107" t="n">
-        <v>26.7703</v>
+        <v>45.3704</v>
       </c>
       <c r="F107" t="n">
-        <v>12.2625</v>
+        <v>7.716</v>
       </c>
     </row>
     <row r="108">
@@ -6756,13 +6756,13 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>24.6224</v>
+        <v>44.7887</v>
       </c>
       <c r="E108" t="n">
-        <v>27.0393</v>
+        <v>45.0704</v>
       </c>
       <c r="F108" t="n">
-        <v>15.71</v>
+        <v>10.1408</v>
       </c>
     </row>
     <row r="109">
@@ -6777,13 +6777,13 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>25.0082</v>
+        <v>46.9343</v>
       </c>
       <c r="E109" t="n">
-        <v>27.0949</v>
+        <v>48.5401</v>
       </c>
       <c r="F109" t="n">
-        <v>8.2165</v>
+        <v>4.5255</v>
       </c>
     </row>
     <row r="110">
@@ -6793,13 +6793,13 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>27.7842</v>
+        <v>47.4747</v>
       </c>
       <c r="E110" t="n">
-        <v>27.3249</v>
+        <v>47.9798</v>
       </c>
       <c r="F110" t="n">
-        <v>8.7256</v>
+        <v>4.5455</v>
       </c>
     </row>
     <row r="111">
@@ -6809,13 +6809,13 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>27.476</v>
+        <v>46.62</v>
       </c>
       <c r="E111" t="n">
-        <v>27.5825</v>
+        <v>49.1841</v>
       </c>
       <c r="F111" t="n">
-        <v>8.626200000000001</v>
+        <v>4.1958</v>
       </c>
     </row>
     <row r="112">
@@ -6830,13 +6830,13 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>28.7066</v>
+        <v>53.6212</v>
       </c>
       <c r="E112" t="n">
-        <v>24.2138</v>
+        <v>38.0117</v>
       </c>
       <c r="F112" t="n">
-        <v>11.0192</v>
+        <v>8.367100000000001</v>
       </c>
     </row>
     <row r="113">
@@ -6846,13 +6846,13 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>28.0754</v>
+        <v>52.037</v>
       </c>
       <c r="E113" t="n">
-        <v>26.1905</v>
+        <v>40.1852</v>
       </c>
       <c r="F113" t="n">
-        <v>11.3095</v>
+        <v>7.7778</v>
       </c>
     </row>
     <row r="114">
@@ -6862,13 +6862,13 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>30.1297</v>
+        <v>55.1674</v>
       </c>
       <c r="E114" t="n">
-        <v>24.18</v>
+        <v>35.6623</v>
       </c>
       <c r="F114" t="n">
-        <v>11.2128</v>
+        <v>9.170299999999999</v>
       </c>
     </row>
     <row r="115">
@@ -6883,13 +6883,13 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>26.3604</v>
+        <v>47.6778</v>
       </c>
       <c r="E115" t="n">
-        <v>27.5249</v>
+        <v>44.7185</v>
       </c>
       <c r="F115" t="n">
-        <v>10.3959</v>
+        <v>7.6038</v>
       </c>
     </row>
     <row r="116">
@@ -6899,13 +6899,13 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>28.9945</v>
+        <v>46.9828</v>
       </c>
       <c r="E116" t="n">
-        <v>26.7342</v>
+        <v>43.9655</v>
       </c>
       <c r="F116" t="n">
-        <v>13.1723</v>
+        <v>9.0517</v>
       </c>
     </row>
     <row r="117">
@@ -6915,13 +6915,13 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>28.0511</v>
+        <v>47.7521</v>
       </c>
       <c r="E117" t="n">
-        <v>27.8594</v>
+        <v>44.593</v>
       </c>
       <c r="F117" t="n">
-        <v>10.7987</v>
+        <v>7.6549</v>
       </c>
     </row>
     <row r="118">
@@ -6936,13 +6936,13 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>26.7978</v>
+        <v>52.9188</v>
       </c>
       <c r="E118" t="n">
-        <v>20.1225</v>
+        <v>36.231</v>
       </c>
       <c r="F118" t="n">
-        <v>12.1251</v>
+        <v>10.8503</v>
       </c>
     </row>
     <row r="119">
@@ -6952,13 +6952,13 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>27.5219</v>
+        <v>53.8627</v>
       </c>
       <c r="E119" t="n">
-        <v>20.614</v>
+        <v>35.6223</v>
       </c>
       <c r="F119" t="n">
-        <v>11.6228</v>
+        <v>10.515</v>
       </c>
     </row>
     <row r="120">
@@ -6968,13 +6968,13 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>27.2095</v>
+        <v>53.831</v>
       </c>
       <c r="E120" t="n">
-        <v>20.4568</v>
+        <v>35.9528</v>
       </c>
       <c r="F120" t="n">
-        <v>12.1152</v>
+        <v>10.2161</v>
       </c>
     </row>
     <row r="121">
@@ -6989,13 +6989,13 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>26.9895</v>
+        <v>52.8999</v>
       </c>
       <c r="E121" t="n">
-        <v>27.0745</v>
+        <v>40.9178</v>
       </c>
       <c r="F121" t="n">
-        <v>10.5919</v>
+        <v>6.1823</v>
       </c>
     </row>
     <row r="122">
@@ -7005,13 +7005,13 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>25.5319</v>
+        <v>48.8414</v>
       </c>
       <c r="E122" t="n">
-        <v>30.6874</v>
+        <v>45.098</v>
       </c>
       <c r="F122" t="n">
-        <v>13.9116</v>
+        <v>6.0606</v>
       </c>
     </row>
     <row r="123">
@@ -7021,13 +7021,13 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>25.2983</v>
+        <v>48.1034</v>
       </c>
       <c r="E123" t="n">
-        <v>30.7876</v>
+        <v>45.5172</v>
       </c>
       <c r="F123" t="n">
-        <v>13.922</v>
+        <v>6.3793</v>
       </c>
     </row>
     <row r="124">
@@ -7042,13 +7042,13 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>27.6178</v>
+        <v>54.7739</v>
       </c>
       <c r="E124" t="n">
-        <v>23.7899</v>
+        <v>39.4831</v>
       </c>
       <c r="F124" t="n">
-        <v>8.6998</v>
+        <v>5.743</v>
       </c>
     </row>
     <row r="125">
@@ -7058,13 +7058,13 @@
         </is>
       </c>
       <c r="D125" t="n">
-        <v>27.1284</v>
+        <v>52.2621</v>
       </c>
       <c r="E125" t="n">
-        <v>24.8196</v>
+        <v>41.4977</v>
       </c>
       <c r="F125" t="n">
-        <v>9.451700000000001</v>
+        <v>6.2402</v>
       </c>
     </row>
     <row r="126">
@@ -7074,13 +7074,13 @@
         </is>
       </c>
       <c r="D126" t="n">
-        <v>27.1899</v>
+        <v>59.4625</v>
       </c>
       <c r="E126" t="n">
-        <v>22.0295</v>
+        <v>34.7144</v>
       </c>
       <c r="F126" t="n">
-        <v>9.757199999999999</v>
+        <v>5.8231</v>
       </c>
     </row>
     <row r="127">
@@ -7095,13 +7095,13 @@
         </is>
       </c>
       <c r="D127" t="n">
-        <v>26.5147</v>
+        <v>49.1598</v>
       </c>
       <c r="E127" t="n">
-        <v>24.3582</v>
+        <v>39.5467</v>
       </c>
       <c r="F127" t="n">
-        <v>12.672</v>
+        <v>11.2935</v>
       </c>
     </row>
     <row r="128">
@@ -7111,13 +7111,13 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>28.1581</v>
+        <v>51.2262</v>
       </c>
       <c r="E128" t="n">
-        <v>23.3592</v>
+        <v>36.6485</v>
       </c>
       <c r="F128" t="n">
-        <v>13.4792</v>
+        <v>12.1253</v>
       </c>
     </row>
     <row r="129">
@@ -7127,13 +7127,13 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>28.1581</v>
+        <v>51.2262</v>
       </c>
       <c r="E129" t="n">
-        <v>23.3592</v>
+        <v>36.6485</v>
       </c>
       <c r="F129" t="n">
-        <v>13.4792</v>
+        <v>12.1253</v>
       </c>
     </row>
     <row r="130">
@@ -7148,13 +7148,13 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>24.4352</v>
+        <v>51.8762</v>
       </c>
       <c r="E130" t="n">
-        <v>23.0678</v>
+        <v>43.318</v>
       </c>
       <c r="F130" t="n">
-        <v>10.2854</v>
+        <v>4.8058</v>
       </c>
     </row>
     <row r="131">
@@ -7164,13 +7164,13 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>21.1329</v>
+        <v>45.5919</v>
       </c>
       <c r="E131" t="n">
-        <v>24.5098</v>
+        <v>48.6146</v>
       </c>
       <c r="F131" t="n">
-        <v>11.4379</v>
+        <v>5.7935</v>
       </c>
     </row>
     <row r="132">
@@ -7180,13 +7180,13 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>22.7556</v>
+        <v>52.1834</v>
       </c>
       <c r="E132" t="n">
-        <v>21.1556</v>
+        <v>42.7948</v>
       </c>
       <c r="F132" t="n">
-        <v>12.7111</v>
+        <v>5.0218</v>
       </c>
     </row>
     <row r="133">
@@ -7201,13 +7201,13 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>25.4825</v>
+        <v>48.6792</v>
       </c>
       <c r="E133" t="n">
-        <v>25.4167</v>
+        <v>41.8449</v>
       </c>
       <c r="F133" t="n">
-        <v>11.9737</v>
+        <v>9.475899999999999</v>
       </c>
     </row>
     <row r="134">
@@ -7217,13 +7217,13 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>27.7604</v>
+        <v>49.9426</v>
       </c>
       <c r="E134" t="n">
-        <v>27.1366</v>
+        <v>42.7095</v>
       </c>
       <c r="F134" t="n">
-        <v>10.6051</v>
+        <v>7.3479</v>
       </c>
     </row>
     <row r="135">
@@ -7233,13 +7233,13 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>27.7431</v>
+        <v>49.9426</v>
       </c>
       <c r="E135" t="n">
-        <v>27.1197</v>
+        <v>42.7095</v>
       </c>
       <c r="F135" t="n">
-        <v>10.5985</v>
+        <v>7.3479</v>
       </c>
     </row>
     <row r="136">
@@ -7254,13 +7254,13 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>28.8809</v>
+        <v>54.2226</v>
       </c>
       <c r="E136" t="n">
-        <v>24.3883</v>
+        <v>39.6212</v>
       </c>
       <c r="F136" t="n">
-        <v>10.5094</v>
+        <v>6.1563</v>
       </c>
     </row>
     <row r="137">
@@ -7270,13 +7270,13 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>29.8851</v>
+        <v>55.3288</v>
       </c>
       <c r="E137" t="n">
-        <v>23.3333</v>
+        <v>37.415</v>
       </c>
       <c r="F137" t="n">
-        <v>13.5632</v>
+        <v>7.2562</v>
       </c>
     </row>
     <row r="138">
@@ -7286,13 +7286,13 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>30.6781</v>
+        <v>56.2372</v>
       </c>
       <c r="E138" t="n">
-        <v>27.2336</v>
+        <v>39.6728</v>
       </c>
       <c r="F138" t="n">
-        <v>10.4413</v>
+        <v>4.09</v>
       </c>
     </row>
     <row r="139">
@@ -7307,13 +7307,13 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>26.011</v>
+        <v>56.3066</v>
       </c>
       <c r="E139" t="n">
-        <v>23.2843</v>
+        <v>40.2787</v>
       </c>
       <c r="F139" t="n">
-        <v>9.436299999999999</v>
+        <v>3.4146</v>
       </c>
     </row>
     <row r="140">
@@ -7323,13 +7323,13 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>25.4394</v>
+        <v>55.0321</v>
       </c>
       <c r="E140" t="n">
-        <v>25.2544</v>
+        <v>42.3983</v>
       </c>
       <c r="F140" t="n">
-        <v>9.9907</v>
+        <v>2.5696</v>
       </c>
     </row>
     <row r="141">
@@ -7339,13 +7339,13 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>26.4922</v>
+        <v>57.7358</v>
       </c>
       <c r="E141" t="n">
-        <v>24.121</v>
+        <v>39.6226</v>
       </c>
       <c r="F141" t="n">
-        <v>10.139</v>
+        <v>2.6415</v>
       </c>
     </row>
     <row r="142">
@@ -7360,13 +7360,13 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>30.0106</v>
+        <v>49.271</v>
       </c>
       <c r="E142" t="n">
-        <v>25.7538</v>
+        <v>42.4666</v>
       </c>
       <c r="F142" t="n">
-        <v>12.5222</v>
+        <v>8.262499999999999</v>
       </c>
     </row>
     <row r="143">
@@ -7376,13 +7376,13 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>29.9043</v>
+        <v>51.2605</v>
       </c>
       <c r="E143" t="n">
-        <v>24.1627</v>
+        <v>40.9664</v>
       </c>
       <c r="F143" t="n">
-        <v>12.201</v>
+        <v>7.7731</v>
       </c>
     </row>
     <row r="144">
@@ -7392,13 +7392,13 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>31.0702</v>
+        <v>49.7992</v>
       </c>
       <c r="E144" t="n">
-        <v>24.5109</v>
+        <v>42.7711</v>
       </c>
       <c r="F144" t="n">
-        <v>13.5788</v>
+        <v>7.4297</v>
       </c>
     </row>
     <row r="145">
@@ -7413,13 +7413,13 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>23.4034</v>
+        <v>51.5362</v>
       </c>
       <c r="E145" t="n">
-        <v>24.8585</v>
+        <v>43.112</v>
       </c>
       <c r="F145" t="n">
-        <v>14.3492</v>
+        <v>5.3518</v>
       </c>
     </row>
     <row r="146">
@@ -7429,13 +7429,13 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>22.0046</v>
+        <v>47.1591</v>
       </c>
       <c r="E146" t="n">
-        <v>26.9585</v>
+        <v>48.8636</v>
       </c>
       <c r="F146" t="n">
-        <v>12.3272</v>
+        <v>3.9773</v>
       </c>
     </row>
     <row r="147">
@@ -7445,13 +7445,13 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>22.0667</v>
+        <v>47.9893</v>
       </c>
       <c r="E147" t="n">
-        <v>26.3724</v>
+        <v>47.7212</v>
       </c>
       <c r="F147" t="n">
-        <v>12.9171</v>
+        <v>4.2895</v>
       </c>
     </row>
     <row r="148">
@@ -7466,13 +7466,13 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>20.674</v>
+        <v>42.1891</v>
       </c>
       <c r="E148" t="n">
-        <v>28.5519</v>
+        <v>50.9453</v>
       </c>
       <c r="F148" t="n">
-        <v>16.1658</v>
+        <v>6.8657</v>
       </c>
     </row>
     <row r="149">
@@ -7482,13 +7482,13 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>18.6608</v>
+        <v>37.1859</v>
       </c>
       <c r="E149" t="n">
-        <v>28.9791</v>
+        <v>55.7789</v>
       </c>
       <c r="F149" t="n">
-        <v>18.112</v>
+        <v>7.0352</v>
       </c>
     </row>
     <row r="150">
@@ -7498,13 +7498,13 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>21.1329</v>
+        <v>42.0538</v>
       </c>
       <c r="E150" t="n">
-        <v>29.085</v>
+        <v>53.3007</v>
       </c>
       <c r="F150" t="n">
-        <v>15.1416</v>
+        <v>4.6455</v>
       </c>
     </row>
     <row r="151">
@@ -7519,13 +7519,13 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>23.9778</v>
+        <v>40.6829</v>
       </c>
       <c r="E151" t="n">
-        <v>28.1984</v>
+        <v>51.0732</v>
       </c>
       <c r="F151" t="n">
-        <v>12.0285</v>
+        <v>8.2439</v>
       </c>
     </row>
     <row r="152">
@@ -7535,13 +7535,13 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>24.6564</v>
+        <v>39.8134</v>
       </c>
       <c r="E152" t="n">
-        <v>29.2955</v>
+        <v>50.8554</v>
       </c>
       <c r="F152" t="n">
-        <v>14.0893</v>
+        <v>9.331300000000001</v>
       </c>
     </row>
     <row r="153">
@@ -7551,13 +7551,13 @@
         </is>
       </c>
       <c r="D153" t="n">
-        <v>24.8082</v>
+        <v>39.8764</v>
       </c>
       <c r="E153" t="n">
-        <v>29.156</v>
+        <v>50.8501</v>
       </c>
       <c r="F153" t="n">
-        <v>13.9812</v>
+        <v>9.2736</v>
       </c>
     </row>
     <row r="154">

</xml_diff>